<commit_message>
- implementation of CONFIG-file with various meta-functions that are useful in INFEED- or OUTFEED-file (see specific description Above each function) - Adjustment of INFEED-file: including a Validation that the crate type from the Excel file is part of the predefined list. - OUTFEED-file: a) Import functions from CONFIG-file, b) adjust class Order to defined columns in the Excel, c)insert new outfeed logic based on 4 stacks and considering stack height (1st draft, must be improved)
</commit_message>
<xml_diff>
--- a/Outfeed_Test.xlsx
+++ b/Outfeed_Test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\eiddpython\eidppython24w-code\lecture_01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\fruit_salad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A4FECD-A02B-43E1-A074-399FC053741E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED7DC52-F335-4C29-8AE2-6C6C78757DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3060" yWindow="3495" windowWidth="21600" windowHeight="11295" xr2:uid="{674A2589-6D5B-4C35-BFDA-084D70AE4967}"/>
+    <workbookView xWindow="2760" yWindow="-15300" windowWidth="21600" windowHeight="11295" xr2:uid="{674A2589-6D5B-4C35-BFDA-084D70AE4967}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -38,18 +38,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
-    <t>OUT-ID</t>
-  </si>
-  <si>
     <t>article_code</t>
   </si>
   <si>
     <t>article_description</t>
   </si>
   <si>
-    <t>OUT-quantity</t>
-  </si>
-  <si>
     <t>shop_destination</t>
   </si>
   <si>
@@ -78,6 +72,12 @@
   </si>
   <si>
     <t>FINOCCHI</t>
+  </si>
+  <si>
+    <t>OUT_ID</t>
+  </si>
+  <si>
+    <t>OUT_quantity</t>
   </si>
 </sst>
 </file>
@@ -458,19 +458,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -478,13 +478,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>20</v>
@@ -495,13 +495,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>40</v>
@@ -512,13 +512,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4">
         <v>40</v>
@@ -529,13 +529,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5">
         <v>10</v>

</xml_diff>